<commit_message>
fix(calculators): treat other livestock nitrogen excreted as per head per year
OTHER_LIVESTOCK_EMISSION_FACTORS.*.NITROGEN_EXCRETED (goats 7, deer 13.2,
horses 39.5 kg N) are annual figures, but were typed as MassPerHeadPerDay
and the 4.7 manure module multiplied them by days in the year. Direct,
atmospheric deposition and leaching N2O from other livestock manure were
365 times too high in both the Other livestock and All-modules calculators.

Type the factor as MassPerHead (kg N per head per year, like ENTERIC),
drop the days term from AE, and update the 4.7 test workbook's AE formula
and cached outputs to match. Add hand-calculated tests for a goat herd and
a mixed herd through All-modules.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/packages/calculators/src/modules/test/4.7-other-livestock-manure/4.7-other-livestock-manure.xlsx
+++ b/packages/calculators/src/modules/test/4.7-other-livestock-manure/4.7-other-livestock-manure.xlsx
@@ -1402,28 +1402,28 @@
         <v>3.0183028512000003E-3</v>
       </c>
       <c r="AE11">
-        <f>C11*P11*365</f>
-        <v>72087.5</v>
+        <f>C11*P11</f>
+        <v>197.5</v>
       </c>
       <c r="AF11">
         <f>AE11*W11*O11*10^-3</f>
-        <v>0.67906425000000015</v>
+        <v>0.0018604500000000003</v>
       </c>
       <c r="AG11">
         <f>AE11*S11</f>
-        <v>15138.375</v>
+        <v>41.475</v>
       </c>
       <c r="AH11">
         <f>AG11*Q11*O11*10^-3</f>
-        <v>0.16637074125000001</v>
+        <v>0.00045581025000000005</v>
       </c>
       <c r="AI11">
         <f>AE11*R11*T11</f>
-        <v>17301</v>
+        <v>47.4</v>
       </c>
       <c r="AJ11">
         <f>AI11*U11*O11*10^-3</f>
-        <v>0.29878826999999997</v>
+        <v>0.000818598</v>
       </c>
       <c r="AM11" s="2" t="s">
         <v>3</v>
@@ -1553,20 +1553,20 @@
         <v>3.6219634214400007E-3</v>
       </c>
       <c r="AE12">
-        <f t="shared" ref="AE12:AE17" si="9">C12*P12*365</f>
-        <v>86505</v>
+        <f t="shared" ref="AE12:AE17" si="9">C12*P12</f>
+        <v>237</v>
       </c>
       <c r="AF12">
         <f t="shared" ref="AF12:AF17" si="10">AE12*W12*O12*10^-3</f>
-        <v>0.81487710000000002</v>
+        <v>0.0022325400000000003</v>
       </c>
       <c r="AG12">
         <f t="shared" ref="AG12:AG17" si="11">AE12*S12</f>
-        <v>18166.05</v>
+        <v>49.769999999999996</v>
       </c>
       <c r="AH12">
         <f t="shared" ref="AH12:AH17" si="12">AG12*Q12*O12*10^-3</f>
-        <v>0.19964488950000001</v>
+        <v>0.0005469723</v>
       </c>
       <c r="AI12">
         <f t="shared" ref="AI12:AI17" si="13">AE12*R12*T12</f>
@@ -1705,27 +1705,27 @@
       </c>
       <c r="AE13">
         <f t="shared" si="9"/>
-        <v>100922.5</v>
+        <v>276.5</v>
       </c>
       <c r="AF13">
         <f t="shared" si="10"/>
-        <v>0.95068995000000001</v>
+        <v>0.00260463</v>
       </c>
       <c r="AG13">
         <f t="shared" si="11"/>
-        <v>21193.724999999999</v>
+        <v>58.065</v>
       </c>
       <c r="AH13">
         <f t="shared" si="12"/>
-        <v>0.19631747467499999</v>
+        <v>0.000537856095</v>
       </c>
       <c r="AI13">
         <f t="shared" si="13"/>
-        <v>24221.399999999998</v>
+        <v>66.36</v>
       </c>
       <c r="AJ13">
         <f t="shared" si="14"/>
-        <v>0.41830357799999995</v>
+        <v>0.0011460372</v>
       </c>
       <c r="AM13" s="2" t="s">
         <v>22</v>
@@ -1856,19 +1856,19 @@
       </c>
       <c r="AE14">
         <f t="shared" si="9"/>
-        <v>115340</v>
+        <v>316</v>
       </c>
       <c r="AF14">
         <f t="shared" si="10"/>
-        <v>1.0865028000000001</v>
+        <v>0.0029767200000000004</v>
       </c>
       <c r="AG14">
         <f t="shared" si="11"/>
-        <v>24221.399999999998</v>
+        <v>66.36</v>
       </c>
       <c r="AH14">
         <f t="shared" si="12"/>
-        <v>0.26619318599999997</v>
+        <v>0.0007292964</v>
       </c>
       <c r="AI14">
         <f t="shared" si="13"/>
@@ -2007,27 +2007,27 @@
       </c>
       <c r="AE15">
         <f t="shared" si="9"/>
-        <v>22995</v>
+        <v>63</v>
       </c>
       <c r="AF15">
         <f t="shared" si="10"/>
-        <v>0.2166129</v>
+        <v>0.00059346</v>
       </c>
       <c r="AG15">
         <f t="shared" si="11"/>
-        <v>4828.95</v>
+        <v>13.229999999999999</v>
       </c>
       <c r="AH15">
         <f t="shared" si="12"/>
-        <v>1.3646612700000001E-2</v>
+        <v>0.00003738798</v>
       </c>
       <c r="AI15">
         <f t="shared" si="13"/>
-        <v>5518.8</v>
+        <v>15.12</v>
       </c>
       <c r="AJ15">
         <f t="shared" si="14"/>
-        <v>9.530967600000001E-2</v>
+        <v>0.0002611224</v>
       </c>
       <c r="AM15" s="2" t="s">
         <v>18</v>
@@ -2158,19 +2158,19 @@
       </c>
       <c r="AE16">
         <f t="shared" si="9"/>
-        <v>25550</v>
+        <v>70</v>
       </c>
       <c r="AF16">
         <f t="shared" si="10"/>
-        <v>0.24068100000000003</v>
+        <v>0.0006594</v>
       </c>
       <c r="AG16">
         <f t="shared" si="11"/>
-        <v>5365.5</v>
+        <v>14.7</v>
       </c>
       <c r="AH16">
         <f t="shared" si="12"/>
-        <v>2.4429121500000001E-2</v>
+        <v>0.00006692909999999999</v>
       </c>
       <c r="AI16">
         <f t="shared" si="13"/>
@@ -2309,27 +2309,27 @@
       </c>
       <c r="AE17">
         <f t="shared" si="9"/>
-        <v>28105</v>
+        <v>77</v>
       </c>
       <c r="AF17">
         <f t="shared" si="10"/>
-        <v>8.82497E-2</v>
+        <v>0.00024178</v>
       </c>
       <c r="AG17">
         <f t="shared" si="11"/>
-        <v>5902.05</v>
+        <v>16.169999999999998</v>
       </c>
       <c r="AH17">
         <f t="shared" si="12"/>
-        <v>7.4129748000000009E-2</v>
+        <v>0.0002030952</v>
       </c>
       <c r="AI17">
         <f t="shared" si="13"/>
-        <v>6745.2</v>
+        <v>18.48</v>
       </c>
       <c r="AJ17">
         <f t="shared" si="14"/>
-        <v>0.116489604</v>
+        <v>0.0003191496</v>
       </c>
       <c r="AM17" s="2" t="s">
         <v>20</v>
@@ -2459,28 +2459,28 @@
         <v>9.7735520896000019E-4</v>
       </c>
       <c r="AE18">
-        <f t="shared" ref="AE18:AE29" si="40">C18*P18*365</f>
-        <v>33215</v>
+        <f t="shared" ref="AE18:AE29" si="40">C18*P18</f>
+        <v>91</v>
       </c>
       <c r="AF18">
         <f t="shared" ref="AF18:AF29" si="41">AE18*W18*O18*10^-3</f>
-        <v>0.10429510000000002</v>
+        <v>0.00028574</v>
       </c>
       <c r="AG18">
         <f t="shared" ref="AG18:AG29" si="42">AE18*S18</f>
-        <v>6975.15</v>
+        <v>19.11</v>
       </c>
       <c r="AH18">
         <f t="shared" ref="AH18:AH29" si="43">AG18*Q18*O18*10^-3</f>
-        <v>7.6656898500000001E-2</v>
+        <v>0.0002100189</v>
       </c>
       <c r="AI18">
         <f t="shared" ref="AI18:AI29" si="44">AE18*R18*T18</f>
-        <v>7971.5999999999995</v>
+        <v>21.84</v>
       </c>
       <c r="AJ18">
         <f t="shared" ref="AJ18:AJ29" si="45">AI18*U18*O18*10^-3</f>
-        <v>0.13766953199999998</v>
+        <v>0.0003771768</v>
       </c>
       <c r="AM18" s="2" t="s">
         <v>62</v>
@@ -2611,19 +2611,19 @@
       </c>
       <c r="AE19">
         <f t="shared" si="40"/>
-        <v>35770</v>
+        <v>98</v>
       </c>
       <c r="AF19">
         <f t="shared" si="41"/>
-        <v>0.11231780000000002</v>
+        <v>0.00030772000000000004</v>
       </c>
       <c r="AG19">
         <f t="shared" si="42"/>
-        <v>7511.7</v>
+        <v>20.58</v>
       </c>
       <c r="AH19">
         <f t="shared" si="43"/>
-        <v>2.1228064200000001E-2</v>
+        <v>0.000058159079999999995</v>
       </c>
       <c r="AI19">
         <f t="shared" si="44"/>
@@ -2753,27 +2753,27 @@
       </c>
       <c r="AE20">
         <f t="shared" si="40"/>
-        <v>38325</v>
+        <v>105</v>
       </c>
       <c r="AF20">
         <f t="shared" si="41"/>
-        <v>0.36102150000000005</v>
+        <v>0.0009891000000000001</v>
       </c>
       <c r="AG20">
         <f t="shared" si="42"/>
-        <v>8048.25</v>
+        <v>22.05</v>
       </c>
       <c r="AH20">
         <f t="shared" si="43"/>
-        <v>3.6643682249999997E-2</v>
+        <v>0.00010039365</v>
       </c>
       <c r="AI20">
         <f t="shared" si="44"/>
-        <v>9198</v>
+        <v>25.2</v>
       </c>
       <c r="AJ20">
         <f t="shared" si="45"/>
-        <v>0.15884946</v>
+        <v>0.00043520400000000007</v>
       </c>
       <c r="AP20" s="2"/>
       <c r="AQ20" s="2"/>
@@ -2895,19 +2895,19 @@
       </c>
       <c r="AE21">
         <f t="shared" si="40"/>
-        <v>77088</v>
+        <v>211.2</v>
       </c>
       <c r="AF21">
         <f t="shared" si="41"/>
-        <v>0.72616896000000009</v>
+        <v>0.001989504</v>
       </c>
       <c r="AG21">
         <f t="shared" si="42"/>
-        <v>16188.48</v>
+        <v>44.352</v>
       </c>
       <c r="AH21">
         <f t="shared" si="43"/>
-        <v>0.2033273088</v>
+        <v>0.0005570611199999999</v>
       </c>
       <c r="AI21">
         <f t="shared" si="44"/>
@@ -3043,27 +3043,27 @@
       </c>
       <c r="AE22">
         <f t="shared" si="40"/>
-        <v>81905.999999999985</v>
+        <v>224.39999999999998</v>
       </c>
       <c r="AF22">
         <f t="shared" si="41"/>
-        <v>0.77155451999999991</v>
+        <v>0.002113848</v>
       </c>
       <c r="AG22">
         <f t="shared" si="42"/>
-        <v>17200.259999999995</v>
+        <v>47.123999999999995</v>
       </c>
       <c r="AH22">
         <f t="shared" si="43"/>
-        <v>0.15932600837999997</v>
+        <v>0.000436509612</v>
       </c>
       <c r="AI22">
         <f t="shared" si="44"/>
-        <v>19657.439999999995</v>
+        <v>53.855999999999995</v>
       </c>
       <c r="AJ22">
         <f t="shared" si="45"/>
-        <v>0.33948398879999991</v>
+        <v>0.0009300931200000001</v>
       </c>
       <c r="AM22" s="2" t="s">
         <v>25</v>
@@ -3186,19 +3186,19 @@
       </c>
       <c r="AE23">
         <f t="shared" si="40"/>
-        <v>86724</v>
+        <v>237.6</v>
       </c>
       <c r="AF23">
         <f t="shared" si="41"/>
-        <v>0.81694008000000007</v>
+        <v>0.0022381920000000004</v>
       </c>
       <c r="AG23">
         <f t="shared" si="42"/>
-        <v>18212.04</v>
+        <v>49.895999999999994</v>
       </c>
       <c r="AH23">
         <f t="shared" si="43"/>
-        <v>0.20015031960000002</v>
+        <v>0.00054835704</v>
       </c>
       <c r="AI23">
         <f t="shared" si="44"/>
@@ -3327,27 +3327,27 @@
       </c>
       <c r="AE24">
         <f t="shared" si="40"/>
-        <v>91542</v>
+        <v>250.79999999999998</v>
       </c>
       <c r="AF24">
         <f t="shared" si="41"/>
-        <v>0.86232564000000012</v>
+        <v>0.002362536</v>
       </c>
       <c r="AG24">
         <f t="shared" si="42"/>
-        <v>19223.82</v>
+        <v>52.66799999999999</v>
       </c>
       <c r="AH24">
         <f t="shared" si="43"/>
-        <v>5.4326515320000004E-2</v>
+        <v>0.000148839768</v>
       </c>
       <c r="AI24">
         <f t="shared" si="44"/>
-        <v>21970.079999999998</v>
+        <v>60.19199999999999</v>
       </c>
       <c r="AJ24">
         <f t="shared" si="45"/>
-        <v>0.37942328159999994</v>
+        <v>0.00103951584</v>
       </c>
       <c r="AM24" s="2" t="s">
         <v>63</v>
@@ -3469,19 +3469,19 @@
       </c>
       <c r="AE25">
         <f t="shared" si="40"/>
-        <v>288350</v>
+        <v>790</v>
       </c>
       <c r="AF25">
         <f t="shared" si="41"/>
-        <v>2.7162570000000006</v>
+        <v>0.007441800000000001</v>
       </c>
       <c r="AG25">
         <f t="shared" si="42"/>
-        <v>60553.5</v>
+        <v>165.9</v>
       </c>
       <c r="AH25">
         <f t="shared" si="43"/>
-        <v>0.27570008550000003</v>
+        <v>0.0007553427</v>
       </c>
       <c r="AI25">
         <f t="shared" si="44"/>
@@ -3611,27 +3611,27 @@
       </c>
       <c r="AE26">
         <f t="shared" si="40"/>
-        <v>53655</v>
+        <v>147</v>
       </c>
       <c r="AF26">
         <f t="shared" si="41"/>
-        <v>0.16847670000000003</v>
+        <v>0.00046158</v>
       </c>
       <c r="AG26">
         <f t="shared" si="42"/>
-        <v>11267.55</v>
+        <v>30.869999999999997</v>
       </c>
       <c r="AH26">
         <f t="shared" si="43"/>
-        <v>0.141520428</v>
+        <v>0.0003877272</v>
       </c>
       <c r="AI26">
         <f t="shared" si="44"/>
-        <v>12877.199999999999</v>
+        <v>35.28</v>
       </c>
       <c r="AJ26">
         <f t="shared" si="45"/>
-        <v>0.22238924399999996</v>
+        <v>0.0006092856</v>
       </c>
       <c r="AM26" s="2" t="s">
         <v>65</v>
@@ -3753,19 +3753,19 @@
       </c>
       <c r="AE27">
         <f t="shared" si="40"/>
-        <v>317185</v>
+        <v>869</v>
       </c>
       <c r="AF27">
         <f t="shared" si="41"/>
-        <v>0.99596090000000004</v>
+        <v>0.00272866</v>
       </c>
       <c r="AG27">
         <f t="shared" si="42"/>
-        <v>66608.849999999991</v>
+        <v>182.48999999999998</v>
       </c>
       <c r="AH27">
         <f t="shared" si="43"/>
-        <v>0.61699777754999996</v>
+        <v>0.00169040487</v>
       </c>
       <c r="AI27">
         <f t="shared" si="44"/>
@@ -3895,27 +3895,27 @@
       </c>
       <c r="AE28">
         <f t="shared" si="40"/>
-        <v>110813.99999999999</v>
+        <v>303.59999999999997</v>
       </c>
       <c r="AF28">
         <f t="shared" si="41"/>
-        <v>0.34795596000000001</v>
+        <v>0.000953304</v>
       </c>
       <c r="AG28">
         <f t="shared" si="42"/>
-        <v>23270.939999999995</v>
+        <v>63.75599999999999</v>
       </c>
       <c r="AH28">
         <f t="shared" si="43"/>
-        <v>0.2557476306</v>
+        <v>0.00070067844</v>
       </c>
       <c r="AI28">
         <f t="shared" si="44"/>
-        <v>26595.359999999997</v>
+        <v>72.86399999999999</v>
       </c>
       <c r="AJ28">
         <f t="shared" si="45"/>
-        <v>0.45930186719999994</v>
+        <v>0.00125836128</v>
       </c>
       <c r="AM28" s="2" t="s">
         <v>67</v>
@@ -4037,19 +4037,19 @@
       </c>
       <c r="AE29">
         <f t="shared" si="40"/>
-        <v>61320</v>
+        <v>168</v>
       </c>
       <c r="AF29">
         <f t="shared" si="41"/>
-        <v>0.19254480000000002</v>
+        <v>0.0005275200000000001</v>
       </c>
       <c r="AG29">
         <f t="shared" si="42"/>
-        <v>12877.199999999999</v>
+        <v>35.28</v>
       </c>
       <c r="AH29">
         <f t="shared" si="43"/>
-        <v>3.6390967199999999E-2</v>
+        <v>0.00009970128000000002</v>
       </c>
       <c r="AI29">
         <f t="shared" si="44"/>

</xml_diff>